<commit_message>
Fix code cho Phat
</commit_message>
<xml_diff>
--- a/src/main/resources/tohop_export.xlsx
+++ b/src/main/resources/tohop_export.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
   <si>
     <t>matohop</t>
   </si>
@@ -41,7 +41,7 @@
     <t>HO</t>
   </si>
   <si>
-    <t>TO - Đã cập nhật</t>
+    <t>Toán, Vật lí, Hóa học</t>
   </si>
   <si>
     <t>A01</t>
@@ -111,15 +111,6 @@
   </si>
   <si>
     <t>Ngữ văn, Năng khiếu âm nhạc</t>
-  </si>
-  <si>
-    <t>A03</t>
-  </si>
-  <si>
-    <t>Toán, Lý, Hóa</t>
-  </si>
-  <si>
-    <t>A04</t>
   </si>
 </sst>
 </file>
@@ -164,14 +155,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="7.76171875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="5.328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="5.328125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="5.328125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="24.02734375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="8.265625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="5.58203125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="5.58203125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="5.58203125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="24.87890625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -327,40 +318,6 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>35</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="C11" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>34</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>